<commit_message>
sync fnomo execution system
</commit_message>
<xml_diff>
--- a/EXCEL/FNOMO_CA_AGGRESSIVE_SCRAPE_86500.xlsx
+++ b/EXCEL/FNOMO_CA_AGGRESSIVE_SCRAPE_86500.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antigravity\eigent\Downloads\fnomo\EXCEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{825DD763-CAAD-4D0A-AA87-8D6B6C93B9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3B89A95-57FE-4CE6-A858-37EE69F7C849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -959,6 +972,7 @@
     <col min="3" max="3" width="9.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.36328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.81640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.08984375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.36328125" bestFit="1" customWidth="1"/>

</xml_diff>